<commit_message>
added Clement's signature to minutes
</commit_message>
<xml_diff>
--- a/Research Logs/Dave/Research Log - Dave.xlsx
+++ b/Research Logs/Dave/Research Log - Dave.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://w2shared-my.sharepoint.com/personal/dave_sushames01_student_wandw_ac_nz/Documents/Documents/Capstone/Research Logs/Dave/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="447" documentId="13_ncr:1_{AF0BDED7-A538-4982-BD37-86F9ACE43960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B606872-97C9-4731-B4C5-BF16F7F083FE}"/>
+  <xr:revisionPtr revIDLastSave="463" documentId="13_ncr:1_{AF0BDED7-A538-4982-BD37-86F9ACE43960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E4849B5-5940-4860-94F5-561D25705936}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="165" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="122">
   <si>
     <t>Date</t>
   </si>
@@ -451,6 +451,24 @@
   </si>
   <si>
     <t>Useful, demonstrates use of magic numbers for file signatures.</t>
+  </si>
+  <si>
+    <t>What parameters can be set for Ais, what are best practices?</t>
+  </si>
+  <si>
+    <t>6 sources found and briefly examined</t>
+  </si>
+  <si>
+    <t>https://www.ibm.com/think/topics/model-parameters</t>
+  </si>
+  <si>
+    <t>https://link.springer.com/article/10.1007/s44163-025-00729-4</t>
+  </si>
+  <si>
+    <t>Not forensics specific, but still solid for genearal Machine Learning.</t>
+  </si>
+  <si>
+    <t>Not particularly useful, seems intended for building an LLM rather than tweaking an existing one's parameters.</t>
   </si>
 </sst>
 </file>
@@ -838,7 +856,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:G68"/>
+  <dimension ref="B2:G72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -857,7 +875,7 @@
       </c>
       <c r="D2" s="4">
         <f>ROUNDDOWN(SUM(C7:C500)/60,0)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>8</v>
@@ -1853,6 +1871,57 @@
         <v>114</v>
       </c>
     </row>
+    <row r="70" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B70" s="2">
+        <v>46281</v>
+      </c>
+      <c r="C70" s="1">
+        <v>10</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="71" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B71" s="2">
+        <v>46281</v>
+      </c>
+      <c r="C71" s="1">
+        <v>20</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="72" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C72" s="1">
+        <v>30</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>